<commit_message>
Bulk Delivered 12 ROs
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -585,7 +585,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>43658486</t>
+          <t>43844458</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -599,19 +599,19 @@
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WCA - Waiting for Approval</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>19/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+          <t>19/9-WCA-In: ,Int: ,Sur: ,Dis: ,App: ,Den: ,Pnt: ,Fit: ,RDY: -Waiting for Approval</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>43844458</t>
+          <t>43809794</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -625,19 +625,19 @@
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>WCA - Waiting for Approval</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>19/9-WCA-In: ,Int: ,Sur: ,Dis: ,App: ,Den: ,Pnt: ,Fit: ,RDY: -Waiting for Approval</t>
+          <t>19/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>43785924</t>
+          <t>44039447</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -651,19 +651,19 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WCA - Waiting for Approval</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve">19/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - PI send </t>
+          <t>19/9-WCA-In: ,Int: ,Sur: ,Dis: ,App: ,Den: ,Pnt: ,Fit: ,RDY: -Waiting for Approval</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>43809794</t>
+          <t>43681230</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -673,61 +673,93 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>19/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>21/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 20/9 - Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>44039447</t>
+          <t>43718251</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>WCA - Waiting for Approval</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>19/9-WCA-In: ,Int: ,Sur: ,Dis: ,App: ,Den: ,Pnt: ,Fit: ,RDY: -Waiting for Approval</t>
+          <t>21/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 20/9 ,App:   - Denting</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>43681230</t>
+          <t>43888271</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -738,44 +770,40 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>21/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 20/9 - Vehicle Ready</t>
+          <t>22/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:22/9,App:22/9,Den:22/9,Pnt:22/9,Fit:22/9-Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>43718251</t>
+          <t>44102135</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>WIP - Denting</t>
+          <t>CASH</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>21/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 20/9 ,App:   - Denting</t>
+          <t>22/9 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>44023023</t>
+          <t>43686750</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -783,29 +811,25 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>21/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 20/9 - Painting</t>
+          <t>22/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>43769098</t>
+          <t>43760706</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -813,83 +837,71 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>22/9 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 22/9 - Vehicle Ready</t>
+          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 21/9 ,Pnt: 23/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>43888271</t>
+          <t>44048543</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>22/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:22/9,App:22/9,Den:22/9,Pnt:22/9,Fit:22/9-Vehicle Ready</t>
+          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 22/9 ,App:   ,Den: 22/9 ,Pnt: 22/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>44102135</t>
+          <t>44145099</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -903,55 +915,91 @@
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>ISP - Claim Intimation Pending</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>22/9 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
+          <t>23/9 - ISP - In:   - Claim Intimation Pending</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>44040772</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>43717479</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>22/9 - IAP - In:   ,Int:   ,Sur: 22/9 ,Dis:   - Approval Pending</t>
+          <t>24/9 - WIP - In: 6/8 ,Int: 7/8 ,Sur: 12/8 ,Dis: 30/8 ,App: 14/8 ,Den:   ,Pnt: 20/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>43686750</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+          <t>43739097</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -959,139 +1007,139 @@
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>22/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
+          <t>24/9 - WIP - In: 8/8 ,Int: 8/8 ,Sur: 11/8 ,Dis:   ,App: 11/8 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>43760706</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+          <t>43902289</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 21/9 ,Pnt: 23/9 - Fitting</t>
+          <t>24/9 - IAP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis:   - investigation</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>44048543</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>44109383</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 22/9 ,App:   ,Den: 22/9 ,Pnt: 22/9 - Fitting</t>
+          <t>24/9 - PNA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>44066357</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+          <t>43689237</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>23/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 22/9 ,App: 22/9 ,Den: 22/9 - Painting</t>
+          <t>24/9 - PNA</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>44091013</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>43686781</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1103,24 +1151,32 @@
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>ISP - Survey Pending</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>23/9 - ISP - In:   ,Int: 23/9 - Survey Pending</t>
+          <t>24/9 - IAP - In: 2/9 ,Int: 2/9 ,Sur:   ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>44145099</t>
+          <t>44070421</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1129,50 +1185,54 @@
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>ISP - Claim Intimation Pending</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>23/9 - ISP - In:   - Claim Intimation Pending</t>
+          <t>24/9 - IAP - In:   ,Int: 21/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>43717479</t>
+          <t>44135014</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1184,34 +1244,22 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 6/8 ,Int: 7/8 ,Sur: 12/8 ,Dis: 30/8 ,App: 14/8 ,Den:   ,Pnt: 20/9 - Fitting</t>
+          <t>24/9 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 22/9 ,Dis: 23/9 ,App: 22/9 ,Den: 23/9 ,Pnt: 24/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>43739097</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
+          <t>44171471</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1221,28 +1269,28 @@
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 8/8 ,Int: 8/8 ,Sur: 11/8 ,Dis:   ,App: 11/8 ,Den:   ,Pnt:   - Fitting</t>
+          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>43883974</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
+          <t>44173725</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1251,106 +1299,126 @@
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>24/9 - RBND - In: 3/9 ,Dis:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready (cashwork)</t>
+          <t>24/9 - IAP - In:   ,Int:   ,Sur: 24/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>43902289</t>
+          <t>43715952</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis:   - investigation</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>43998631</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>43739478</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In:   ,Int: 22/9 ,Sur: 22/9 - Dismantle</t>
+          <t>28/9-RBND-In:11/9,Int:11/9,Sur:12/9,Dis: ,App:14/9,Den:22/9,Pnt:28/9,Fit: -Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>44109383</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+          <t>43849704</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
@@ -1361,113 +1429,129 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>24/9 - PNA</t>
+          <t>28/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>43689237</t>
+          <t>43877087</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>24/9 - PNA</t>
+          <t>28/9 - WIP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>44011687</t>
+          <t>44004899</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den:   ,Pnt: 20/9 - Fitting</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>43686781</t>
+          <t>44076603</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -1480,36 +1564,48 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In: 2/9 ,Int: 2/9 ,Sur:   ,Dis:   - Approval Pending</t>
+          <t>28/9 - IAP - In: 21/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>43732625</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+          <t>44108850</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
@@ -1518,25 +1614,25 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>24/9 - RBND - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit:   - Vehicle Ready</t>
+          <t>28/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:23/9,App:23/9,Den:23/9,Pnt: ,Fit:28/9-Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>44070421</t>
+          <t>44260223</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1552,76 +1648,68 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In:   ,Int: 21/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
+          <t>28/9 - IAP - In:   ,Int: 26/9 ,Sur: 27/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>44135014</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>43655880</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 22/9 ,Dis: 23/9 ,App: 22/9 ,Den: 23/9 ,Pnt: 24/9 - Fitting</t>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur: 20/9 - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>44163447</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
+          <t>43787390</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -1631,229 +1719,225 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>44171471</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+          <t>43819129</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>28/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den: 27/9 - Painting</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>44173725</t>
+          <t>43938356</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In:   ,Int:   ,Sur: 24/9 ,Dis:   - Approval Pending</t>
+          <t>28/9-RBND-In: ,Int: ,Sur: ,Dis: ,App:22/9,Den:27/9,Pnt:27/9,Fit:28/9-Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>43715952</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
+          <t>44072159</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
           <t>2026-09-27</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 27/9 ,App:   - Denting</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>43739478</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>43931687</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>28/9-RBND-In:11/9,Int:11/9,Sur:12/9,Dis: ,App:14/9,Den:22/9,Pnt:28/9,Fit: -Vehicle Ready</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>43849704</t>
+          <t>44049849</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>28/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim</t>
+          <t>28/9-RBND-In: ,Int: ,Sur:21/9,Dis: ,App:22/9,Den:24/9,Pnt:26/9,Fit:28/9-Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>43877087</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+          <t>44050017</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1861,89 +1945,81 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 - Dismantle</t>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 21/9 ,App: 21/9 ,Den: 22/9 ,Pnt: 27/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>44004899</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
+          <t>44050137</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 28/9 ,App: 24/9 ,Den: 28/9 - Painting</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>44076603</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
+          <t>44146209</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
@@ -1951,83 +2027,79 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>PNA</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>28/9 - IAP - In: 21/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Approval Pending</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>44108850</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
+          <t>44210428</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:23/9,App:23/9,Den:23/9,Pnt: ,Fit:28/9-Vehicle Ready</t>
+          <t>28/9 - IAP - In: 25/9 ,Int: 26/9 ,Sur: 27/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>44260223</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t>44241320</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
@@ -2035,73 +2107,89 @@
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>28/9 - IAP - In:   ,Int: 26/9 ,Sur: 27/9 ,Dis:   - Approval Pending</t>
+          <t>28/9 - WIP - In: 24/9 ,Int: 25/9 ,Sur: 25/9 ,Dis:   ,App: 28/9 - Denting</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>43655880</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
+          <t>43739311</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur: 20/9 - Dismantle</t>
+          <t>29/9 - WIP - In: 3/9 ,Int: 3/9 ,Sur: 3/9 ,Dis:   ,App: 9/9 ,Den: 28/9 ,Pnt: 29/9 - Fitting</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>43787390</t>
+          <t>43998801</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2111,41 +2199,29 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>29/9 - IAP - In: 18/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>43819129</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+          <t>44228604</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -2158,102 +2234,94 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den: 27/9 - Painting</t>
+          <t>29/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 29/9 - Painting</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>43938356</t>
+          <t>44261809</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int: ,Sur: ,Dis: ,App:22/9,Den:27/9,Pnt:27/9,Fit:28/9-Vehicle Ready</t>
+          <t>29/9 - IAP - In:   ,Int: 28/9 ,Sur: 29/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>44072159</t>
+          <t>44260904</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>WIP - Denting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 27/9 ,App:   - Denting</t>
+          <t xml:space="preserve">29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim </t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>43931687</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
+          <t>43794910</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
@@ -2264,154 +2332,166 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>29/9 - PNA - Part not available</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>44049849</t>
+          <t>44044061</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int: ,Sur:21/9,Dis: ,App:22/9,Den:24/9,Pnt:26/9,Fit:28/9-Vehicle Ready</t>
+          <t>29/9 - WIP - In:   ,Int:   ,Sur: 20/9 ,Dis:   ,App: 25/9 ,Den: 29/9 - Painting</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>44050017</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
+          <t>44274626</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 21/9 ,App: 21/9 ,Den: 22/9 ,Pnt: 27/9 - Fitting</t>
+          <t>29/9 - WIP - In: 28/9 ,Int: 28/9 ,Sur: 28/9 ,Dis: 29/9 ,App: 29/9 ,Den: 29/9 - Painting</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>44050137</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
+          <t>43809445</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 28/9 ,App: 24/9 ,Den: 28/9 - Painting</t>
+          <t>29/9 - WIP - In: 1/6 ,Int: 1/6 ,Sur: 2/6 ,Dis:   ,App: 22/6 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>44146209</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
+          <t>43810667</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
@@ -2419,37 +2499,41 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>29/9 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 21/8 ,Dis:   ,App: 25/8 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>44210428</t>
+          <t>43857886</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -2462,36 +2546,32 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>28/9 - IAP - In: 25/9 ,Int: 26/9 ,Sur: 27/9 ,Dis:   - Approval Pending</t>
+          <t>29/9 - IAP - In: 14/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Investigation</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>44241320</t>
+          <t>44044364</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
@@ -2499,508 +2579,36 @@
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
-          <t>WIP - Denting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In: 24/9 ,Int: 25/9 ,Sur: 25/9 ,Dis:   ,App: 28/9 - Denting</t>
+          <t>29/9 - IAP - In: 19/9 ,Int: 20/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>43739311</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
+          <t>44089995</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In: 3/9 ,Int: 3/9 ,Sur: 3/9 ,Dis:   ,App: 9/9 ,Den: 28/9 ,Pnt: 29/9 - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>43998801</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>29/9 - IAP - In: 18/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Approval Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>44228604</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>WIP - Painting</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 29/9 - Painting</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>44261809</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>29/9 - IAP - In:   ,Int: 28/9 ,Sur: 29/9 ,Dis:   - Approval Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>44260904</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim </t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>43794910</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>PNA</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>29/9 - PNA - Part not available</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>44044061</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>WIP - Painting</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In:   ,Int:   ,Sur: 20/9 ,Dis:   ,App: 25/9 ,Den: 29/9 - Painting</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>44274626</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>WIP - Painting</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In: 28/9 ,Int: 28/9 ,Sur: 28/9 ,Dis: 29/9 ,App: 29/9 ,Den: 29/9 - Painting</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>43809445</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>WIP - Fitting</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In: 1/6 ,Int: 1/6 ,Sur: 2/6 ,Dis:   ,App: 22/6 ,Den:   ,Pnt:   - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>43810667</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>WIP - Fitting</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>29/9 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 21/8 ,Dis:   ,App: 25/8 ,Den:   ,Pnt:   - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>43857886</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>29/9 - IAP - In: 14/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Investigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>44044364</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>29/9 - IAP - In: 19/9 ,Int: 20/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>44089995</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>IAP - Approval Pending</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
         <is>
           <t>29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - TPFE Affidavit/ Approval pending</t>
         </is>

</xml_diff>

<commit_message>
Bulk Delivered 17 ROs
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R81"/>
+  <dimension ref="A1:R64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -711,72 +711,44 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>43888271</t>
+          <t>44102135</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>22/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:22/9,App:22/9,Den:22/9,Pnt:22/9,Fit:22/9-Vehicle Ready</t>
+          <t>22/9 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>CASH</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>44102135</t>
+          <t>43760706</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>22/9 - WIP - In:   ,Dis:   ,Den:   ,Pnt:   - Fitting (cashwork)</t>
+          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 21/9 ,Pnt: 23/9 - Fitting</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -788,27 +760,35 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>43760706</t>
+          <t>44145099</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 21/9 ,Pnt: 23/9 - Fitting</t>
+          <t>23/9 - ISP - In:   - Claim Intimation Pending</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -820,60 +800,56 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>ISP - Claim Intimation Pending</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>44048543</t>
+          <t>43739097</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>23/9 - WIP - In:   ,Int:   ,Sur:   ,Dis: 22/9 ,App:   ,Den: 22/9 ,Pnt: 22/9 - Fitting</t>
+          <t>24/9 - WIP - In: 8/8 ,Int: 8/8 ,Sur: 11/8 ,Dis:   ,App: 11/8 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
@@ -887,12 +863,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>44145099</t>
+          <t>44173725</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23/9 - ISP - In:   - Claim Intimation Pending</t>
+          <t>24/9 - IAP - In:   ,Int:   ,Sur: 24/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -900,7 +876,11 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -912,44 +892,28 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ISP - Claim Intimation Pending</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>43739097</t>
+          <t>43849704</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 8/8 ,Int: 8/8 ,Sur: 11/8 ,Dis:   ,App: 11/8 ,Den:   ,Pnt:   - Fitting</t>
+          <t>28/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -960,19 +924,19 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>43902289</t>
+          <t>44004899</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis:   - investigation</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -980,22 +944,22 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1008,19 +972,19 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>PNA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>43689237</t>
+          <t>43787390</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>24/9 - PNA</t>
+          <t>28/9 - PNA - Part not available</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -1028,20 +992,24 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -1059,83 +1027,67 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>44135014</t>
+          <t>44260904</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 22/9 ,Dis: 23/9 ,App: 22/9 ,Den: 23/9 ,Pnt: 24/9 - Fitting</t>
+          <t xml:space="preserve">29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim </t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>44171471</t>
+          <t>43857886</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>24/9 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>29/9 - IAP - In: 14/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Investigation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1148,29 +1100,37 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>44173725</t>
+          <t>44044364</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>24/9 - IAP - In:   ,Int:   ,Sur: 24/9 ,Dis:   - Approval Pending</t>
+          <t>29/9 - IAP - In: 19/9 ,Int: 20/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -1191,12 +1151,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>43739478</t>
+          <t>43998801</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28/9-RBND-In:11/9,Int:11/9,Sur:12/9,Dis: ,App:14/9,Den:22/9,Pnt:28/9,Fit: -Vehicle Ready</t>
+          <t>30/9 - WIP - In: 18/9 ,Int: 21/9 ,Sur: 21/9 - Dismantle</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1204,87 +1164,99 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>43849704</t>
+          <t>43819129</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim</t>
+          <t>30/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den: 27/9 ,Pnt: 30/9 - Fitting</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>44004899</t>
+          <t>43715952</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>5/10 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 18/8 ,Dis: 21/9 ,App: 25/8 ,Den: 21/9 ,Pnt: 27/9 - Fitting</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1292,83 +1264,99 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>44108850</t>
+          <t>43717479</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int:22/9,Sur:22/9,Dis:23/9,App:23/9,Den:23/9,Pnt: ,Fit:28/9-Vehicle Ready</t>
+          <t>5/10-RBND-In:6/8,Int:7/8,Sur:12/8,Dis:30/8,App:14/8,Den: ,Pnt:20/9,Fit:4/10-DO awaited</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O22" t="inlineStr"/>
@@ -1383,40 +1371,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>43787390</t>
+          <t>43721281</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 3/10 - Painting</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
@@ -1424,47 +1400,59 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>43938356</t>
+          <t>43739311</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int: ,Sur: ,Dis: ,App:22/9,Den:27/9,Pnt:27/9,Fit:28/9-Vehicle Ready</t>
+          <t>5/10-RBND-In:3/9,Int:3/9,Sur:3/9,Dis: ,App:9/9,Den:28/9,Pnt:29/9,Fit:4/10-Vehicle Ready</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
@@ -1479,21 +1467,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>43931687</t>
+          <t>43877087</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>5/10 - WIP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis: 21/9 ,App: 18/9 ,Den: 4/10 ,Pnt: 5/10 - Fitting</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
@@ -1502,36 +1506,48 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>44049849</t>
+          <t>44076603</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28/9-RBND-In: ,Int: ,Sur:21/9,Dis: ,App:22/9,Den:24/9,Pnt:26/9,Fit:28/9-Vehicle Ready</t>
+          <t>5/10 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   ,App: 3/10 ,Den: 5/10 - Painting</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>2026-09-21</t>
@@ -1539,96 +1555,72 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>44050017</t>
+          <t>44109383</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 21/9 ,App: 21/9 ,Den: 22/9 ,Pnt: 27/9 - Fitting</t>
+          <t>5/10 - WIP - In: 22/9 ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   - Painting</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>44050137</t>
+          <t>44228604</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>28/9 - WIP - In:   ,Int:   ,Sur: 21/9 ,Dis: 28/9 ,App: 24/9 ,Den: 28/9 - Painting</t>
+          <t>5/10 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 29/9 ,Pnt: 30/9 ,Fit: 5/10 - Vehicle Ready</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1636,56 +1628,64 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>44146209</t>
+          <t>44260223</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>28/9 - PNA - Part not available</t>
+          <t>5/10 - WIP - In:   ,Int: 26/9 ,Sur: 27/9 - Dismantle</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
@@ -1696,28 +1696,40 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>PNA</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>44260904</t>
+          <t>44261809</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">29/9 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - No Claim </t>
+          <t>5/10 - WIP - In:   ,Int: 28/9 ,Sur: 29/9 - Dismantle</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -1728,55 +1740,31 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>44274626</t>
+          <t>44261876</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>29/9 - WIP - In: 28/9 ,Int: 28/9 ,Sur: 28/9 ,Dis: 29/9 ,App: 29/9 ,Den: 29/9 - Painting</t>
+          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - claim withdrawl</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
@@ -1784,44 +1772,28 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>43809445</t>
+          <t>44406352</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>29/9 - WIP - In: 1/6 ,Int: 1/6 ,Sur: 2/6 ,Dis:   ,App: 22/6 ,Den:   ,Pnt:   - Fitting</t>
+          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -1832,47 +1804,39 @@
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>43810667</t>
+          <t>44163189</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>29/9 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 21/8 ,Dis:   ,App: 25/8 ,Den:   ,Pnt:   - Fitting</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis: 5/10 ,App:   ,Den: 5/10 - Painting</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
@@ -1880,19 +1844,19 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>43857886</t>
+          <t>44210428</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>29/9 - IAP - In: 14/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   - Investigation</t>
+          <t>5/10 - WIP - In: 25/9 ,Int: 26/9 ,Sur: 27/9 ,Dis:   ,App: 4/10 - Denting</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1900,22 +1864,22 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -1928,19 +1892,19 @@
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>44044364</t>
+          <t>44241320</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>29/9 - IAP - In: 19/9 ,Int: 20/9 ,Sur: 22/9 ,Dis:   - Approval Pending</t>
+          <t>5/10 - WIP - In: 24/9 ,Int: 25/9 ,Sur: 25/9 - Dismantle</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1948,20 +1912,24 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr"/>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -1972,42 +1940,30 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>43998801</t>
+          <t>44381985</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>30/9 - WIP - In: 18/9 ,Int: 21/9 ,Sur: 21/9 - Dismantle</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -2027,200 +1983,140 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>43819129</t>
+          <t>43844458</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>30/9 - WIP - In: 2/9 ,Int: 2/9 ,Sur: 2/9 ,Dis:   ,App:   ,Den: 27/9 ,Pnt: 30/9 - Fitting</t>
+          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>43715952</t>
+          <t>44356089</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 18/8 ,Int: 18/8 ,Sur: 18/8 ,Dis: 21/9 ,App: 25/8 ,Den: 21/9 ,Pnt: 27/9 - Fitting</t>
+          <t>5/10 - IAP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>43717479</t>
+          <t>44439233</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>5/10-RBND-In:6/8,Int:7/8,Sur:12/8,Dis:30/8,App:14/8,Den: ,Pnt:20/9,Fit:4/10-DO awaited</t>
+          <t>5/10 - ISP - In:   ,Int: 4/10 - Survey Pending</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>ISP - Survey Pending</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>43721281</t>
+          <t>44445402</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 3/10 - Painting</t>
+          <t>5/10 - IAP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   - Approval Pending</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
@@ -2228,19 +2124,19 @@
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>43739311</t>
+          <t>43809794</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5/10-RBND-In:3/9,Int:3/9,Sur:3/9,Dis: ,App:9/9,Den:28/9,Pnt:29/9,Fit:4/10-Vehicle Ready</t>
+          <t>5/10 - WIP - In: 27/8 ,Int: 3/9 ,Sur: 4/9 ,Dis:   ,App: 7/9 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -2248,119 +2144,83 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>43877087</t>
+          <t>44089995</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 16/9 ,Int: 16/9 ,Sur: 16/9 ,Dis: 21/9 ,App: 18/9 ,Den: 4/10 ,Pnt: 5/10 - Fitting</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>44076603</t>
+          <t>44416078</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 21/9 ,Int: 21/9 ,Sur: 21/9 ,Dis:   ,App: 3/10 ,Den: 5/10 - Painting</t>
+          <t>5/10 - WIP - In: 14/9 ,Int: 15/9 ,Sur: 17/9 - Dismantle</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -2368,17 +2228,17 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2388,11 +2248,7 @@
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr"/>
@@ -2400,19 +2256,19 @@
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>44109383</t>
+          <t>43686781</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 22/9 ,Int:   ,Sur:   ,Dis:   ,App:   ,Den:   - Painting</t>
+          <t>5/10 - IAP - In: 2/9 ,Int: 2/9 ,Sur:   ,Dis:   - Approval Pending     Ticket - CAS-96437-G3P1J5</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -2420,10 +2276,14 @@
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
@@ -2436,19 +2296,19 @@
       <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>44228604</t>
+          <t>43686750</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>5/10 - RBND - In:   ,Int:   ,Sur:   ,Dis:   ,App:   ,Den: 29/9 ,Pnt: 30/9 ,Fit: 5/10 - Vehicle Ready</t>
+          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending    Ticket - CAS-96436-J8J0F0</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -2460,62 +2320,50 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
       <c r="Q45" t="inlineStr"/>
       <c r="R45" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
+          <t>IAP - Approval Pending</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>44260223</t>
+          <t>43655880</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int: 26/9 ,Sur: 27/9 - Dismantle</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur: 20/9 ,Dis: 3/10 ,App: 27/9 - Denting</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
         <is>
           <t>2026-10-03</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -2524,63 +2372,71 @@
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>44261809</t>
+          <t>44044061</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int: 28/9 ,Sur: 29/9 - Dismantle</t>
+          <t>5/10-RBND-In: ,Int: ,Sur:20/9,Dis: ,App:25/9,Den:29/9,Pnt:4/10,Fit:5/10-Vehicle Ready</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
       <c r="R47" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>44261876</t>
+          <t>44072159</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - claim withdrawl</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis: 27/9 ,App:   - chassis repair</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2591,7 +2447,11 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
@@ -2600,19 +2460,19 @@
       <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>44406352</t>
+          <t>44376284</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
+          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App: 3/10 ,Den:   ,Pnt:   - Fitting</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2621,7 +2481,11 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -2632,39 +2496,35 @@
       <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>44163189</t>
+          <t>44438700</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis: 5/10 ,App:   ,Den: 5/10 - Painting</t>
+          <t>5/10 - ISP - In:   ,Int: 5/10 - Survey Pending</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
@@ -2672,42 +2532,38 @@
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
-          <t>WIP - Painting</t>
+          <t>ISP - Survey Pending</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>44210428</t>
+          <t>44439724</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 25/9 ,Int: 26/9 ,Sur: 27/9 ,Dis:   ,App: 4/10 - Denting</t>
+          <t>5/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   ,App: 5/10 - Denting</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J51" t="inlineStr"/>
@@ -2727,12 +2583,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>44241320</t>
+          <t>43794910</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 24/9 ,Int: 25/9 ,Sur: 25/9 - Dismantle</t>
+          <t>6/10 - RBND - In: 1/9 ,Int: 1/9 ,Sur: 1/9 ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 6/10 - Vehicle Ready</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -2740,95 +2596,139 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>44381985</t>
+          <t>44437107</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>6/10-RBND-In: ,Int:5/10,Sur:6/10,Dis:6/10,App:6/10,Den:6/10,Pnt:6/10,Fit:6/10-Vehicle Ready</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>RBND - Vehicle Ready</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>43844458</t>
+          <t>44438146</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending</t>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 6/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 - Painting</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
       <c r="O54" t="inlineStr"/>
@@ -2836,19 +2736,19 @@
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>44356089</t>
+          <t>44479958</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   - Approval Pending</t>
+          <t>6/10 - WIP - In:   ,Int: 6/10 ,Sur: 6/10 ,Dis: 6/10 ,App:   ,Den: 6/10 - Painting</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -2857,18 +2757,26 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
@@ -2876,30 +2784,26 @@
       <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Painting</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>44439233</t>
+          <t>44483511</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>5/10 - ISP - In:   ,Int: 4/10 - Survey Pending</t>
+          <t>6/10 - PNA - Part not available</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
@@ -2912,35 +2816,27 @@
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
-          <t>ISP - Survey Pending</t>
+          <t>PNA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>44445402</t>
+          <t>44163778</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   - Approval Pending</t>
+          <t>6/10 - PNA - Part not available</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
@@ -2952,78 +2848,82 @@
       <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>PNA</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>43809794</t>
+          <t>44485422</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 27/8 ,Int: 3/9 ,Sur: 4/9 ,Dis:   ,App: 7/9 ,Den:   ,Pnt:   - Fitting</t>
+          <t>6/10 - WIP - In:   ,Dis: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting (cashwork)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
       <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
-          <t>WIP - Fitting</t>
+          <t>CASH</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>44089995</t>
+          <t>44070421</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   - Dismantle</t>
+          <t>6/10 - WIP - In:   ,Int: 21/9 ,Sur: 22/9 - Dismantle</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -3043,79 +2943,95 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>44416078</t>
+          <t>44437682</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In: 14/9 ,Int: 15/9 ,Sur: 17/9 - Dismantle</t>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
-          <t>WIP - Dismantle</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>43686781</t>
+          <t>44439791</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In: 2/9 ,Int: 2/9 ,Sur:   ,Dis:   - Approval Pending     Ticket - CAS-96437-G3P1J5</t>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 5/10 - Denting</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
@@ -3124,74 +3040,98 @@
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Denting</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>43686750</t>
+          <t>44452638</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>5/10 - IAP - In:   ,Int:   ,Sur:   ,Dis:   - Approval Pending    Ticket - CAS-96436-J8J0F0</t>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 5/10 ,App: 5/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr">
         <is>
-          <t>IAP - Approval Pending</t>
+          <t>WIP - Fitting</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>43655880</t>
+          <t>44455086</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur: 20/9 ,Dis: 3/10 ,App: 27/9 - Denting</t>
+          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 - Dismantle</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
+      <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
@@ -3200,814 +3140,46 @@
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr">
         <is>
-          <t>WIP - Denting</t>
+          <t>WIP - Dismantle</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>44044061</t>
+          <t>44366447</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>5/10-RBND-In: ,Int: ,Sur:20/9,Dis: ,App:25/9,Den:29/9,Pnt:4/10,Fit:5/10-Vehicle Ready</t>
+          <t>6/10 - IAP - In:   ,Int: 5/10 ,Sur: 4/10 ,Dis:   - Approval Pending    Ticket - CAS-96544-S5W5G9</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr">
         <is>
-          <t>RBND - Vehicle Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>44072159</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis: 27/9 ,App:   - chassis repair</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>WIP - Denting</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>44376284</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>5/10 - WIP - In:   ,Int:   ,Sur:   ,Dis:   ,App: 3/10 ,Den:   ,Pnt:   - Fitting</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>WIP - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>44438700</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>5/10 - ISP - In:   ,Int: 5/10 - Survey Pending</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>ISP - Survey Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>44439724</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>5/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis:   ,App: 5/10 - Denting</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>WIP - Denting</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>43794910</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>6/10 - RBND - In: 1/9 ,Int: 1/9 ,Sur: 1/9 ,Dis:   ,App:   ,Den:   ,Pnt:   ,Fit: 6/10 - Vehicle Ready</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>RBND - Vehicle Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>44437107</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>6/10-RBND-In: ,Int:5/10,Sur:6/10,Dis:6/10,App:6/10,Den:6/10,Pnt:6/10,Fit:6/10-Vehicle Ready</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>RBND - Vehicle Ready</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>44438146</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 6/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 - Painting</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>WIP - Painting</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>44479958</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 6/10 ,Sur: 6/10 ,Dis: 6/10 ,App:   ,Den: 6/10 - Painting</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>WIP - Painting</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>44483511</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>6/10 - PNA - Part not available</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
-      <c r="Q73" t="inlineStr"/>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>PNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>44163778</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>6/10 - PNA - Part not available</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
-      <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="inlineStr"/>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>PNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>44485422</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Dis: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting (cashwork)</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
-      <c r="P75" t="inlineStr"/>
-      <c r="Q75" t="inlineStr"/>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>CASH</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>44070421</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 21/9 ,Sur: 22/9 - Dismantle</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>WIP - Dismantle</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>44437682</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 6/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
-      <c r="Q77" t="inlineStr"/>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>WIP - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>44439791</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 6/10 ,App: 5/10 - Denting</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
-      <c r="P78" t="inlineStr"/>
-      <c r="Q78" t="inlineStr"/>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>WIP - Denting</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>44452638</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 ,Dis: 5/10 ,App: 5/10 ,Den: 6/10 ,Pnt: 6/10 - Fitting</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr"/>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
-      <c r="P79" t="inlineStr"/>
-      <c r="Q79" t="inlineStr"/>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>WIP - Fitting</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>44455086</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>6/10 - WIP - In:   ,Int: 5/10 ,Sur: 5/10 - Dismantle</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr"/>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>WIP - Dismantle</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>44366447</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>6/10 - IAP - In:   ,Int: 5/10 ,Sur: 4/10 ,Dis:   - Approval Pending    Ticket - CAS-96544-S5W5G9</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr">
-        <is>
           <t>IAP - Approval Pending</t>
         </is>
       </c>

</xml_diff>